<commit_message>
recon-app: update data/Unmatched_History.xlsx [2026-03-18 04:27 UTC]
</commit_message>
<xml_diff>
--- a/data/Unmatched_History.xlsx
+++ b/data/Unmatched_History.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,6 +694,255 @@
       </c>
       <c r="S3" s="2" t="n">
         <v>46098</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46095.71125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46095.71127314815</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Settlement_Direct_Debit</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>be4480e0-0b91-4714-98e1-7976c461368f</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>BUS/MRT 813134050        SINGAPORE    SG</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>FR6065SDD</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>FR6065SDD</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FR6065SDD</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>AMAZE</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>nan_1.75</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Pending Transactions</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>46099</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46095.71342592593</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46095.71347222223</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Settlement_Debit</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>30909667-1441-4ed4-b563-fed59a34a6f8</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>BUS/MRT                  SINGAPORE    SG</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ESJ60NSD</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>922488SD</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>707996      SD</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>AMAZE</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>nan_14.35</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Pending Transactions</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>46099</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46096.71350694444</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46096.71354166666</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Settlement_Debit</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>31222f56-f894-4c73-9e59-ce35c2809afa</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BUS/MRT                  SINGAPORE    SG</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>YBD1IESD</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>236587SD</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>743872      SD</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>AMAZE</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>nan_7.6</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Pending Transactions</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>46099</v>
       </c>
     </row>
   </sheetData>
@@ -707,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1018,6 +1267,154 @@
       </c>
       <c r="P4" s="2" t="n">
         <v>46098</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AMAZEMCAP</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46096.06287037037</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sgd</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>247.03</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>charge</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ch_3TB3VjC9gcIngfzT1Jc9IIWe</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>pi_3TB3VjC9gcIngfzT1fduw4Lt</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>606806085836SDD</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>085836SDD</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>UNIQLO CO.,LTD</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>pi_3TB3VjC9gcIngfzT1fduw4Lt_247.03</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>ch_3TB3VjC9gcIngfzT1Jc9IIWe_247.03</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>pi_3TB3VjC9gcIngfzT1fduw4Lt_247.03</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Need to Investigate</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>46099</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AMAZEMCREST</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46095.60791666667</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>sgd</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2390.81</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>refund</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>re_3SrK8ZLoUHgGqMC50DfJHmLX</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>pi_3SrK8ZLoUHgGqMC50QHWxrpm</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>601915616886</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>616886</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PAYPAL *HOME DEPOT</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>pi_3SrK8ZLoUHgGqMC50QHWxrpm_2390.81</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>re_3SrK8ZLoUHgGqMC50DfJHmLX_2390.81</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Dispute Write Off/Chargeback Credit</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>46099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>